<commit_message>
fix bug- hif genen as sasp
</commit_message>
<xml_diff>
--- a/Reports/Bulk/03_bulk_cell_lines_march25/04_GSVA/GSVA_scores_heatmap.xlsx
+++ b/Reports/Bulk/03_bulk_cell_lines_march25/04_GSVA/GSVA_scores_heatmap.xlsx
@@ -2746,44 +2746,44 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>SASP</t>
+          <t>KAMMINGA_SENESCENCE</t>
         </is>
       </c>
       <c r="B56">
-        <v>0.1170590355197069</v>
+        <v>1.111027647118721</v>
       </c>
       <c r="C56">
-        <v>1.068769106204408</v>
+        <v>-0.2975745441466948</v>
       </c>
       <c r="D56">
-        <v>-1.222297930987141</v>
+        <v>1.361458043616241</v>
       </c>
       <c r="E56">
-        <v>0.8666114736016001</v>
+        <v>-0.7280439805049908</v>
       </c>
       <c r="F56">
-        <v>-1.207041325683225</v>
+        <v>-0.3721939086084353</v>
       </c>
       <c r="G56">
-        <v>0.3768996413446511</v>
+        <v>-1.074673257474841</v>
       </c>
       <c r="H56">
-        <v>-0.5273678909157152</v>
+        <v>1.471225630556525</v>
       </c>
       <c r="I56">
-        <v>0.9386386930518482</v>
+        <v>-0.405441963113315</v>
       </c>
       <c r="J56">
-        <v>-1.032453551811761</v>
+        <v>0.7292611432843187</v>
       </c>
       <c r="K56">
-        <v>1.081862413258717</v>
+        <v>-0.7714059982495033</v>
       </c>
       <c r="L56">
-        <v>-1.09588619607448</v>
+        <v>0.202430102019481</v>
       </c>
       <c r="M56">
-        <v>0.6352065324913916</v>
+        <v>-1.226068914497507</v>
       </c>
     </row>
     <row r="57">
@@ -2875,44 +2875,44 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>GOBP_POSITIVE_REGULATION_OF_CELLULAR_SENESCENCE</t>
+          <t>SASP</t>
         </is>
       </c>
       <c r="B59">
-        <v>-1.364787107537137</v>
+        <v>-0.9669076012671058</v>
       </c>
       <c r="C59">
-        <v>-0.8708796600129045</v>
+        <v>-1.146543938812737</v>
       </c>
       <c r="D59">
-        <v>0.1049892474647002</v>
+        <v>-0.4363686918971418</v>
       </c>
       <c r="E59">
-        <v>1.364819788231777</v>
+        <v>0.3635830417593641</v>
       </c>
       <c r="F59">
-        <v>0.708428435607024</v>
+        <v>1.231140146895716</v>
       </c>
       <c r="G59">
-        <v>0.05742929624654035</v>
+        <v>0.9550970433219047</v>
       </c>
       <c r="H59">
-        <v>-0.6304846717014383</v>
+        <v>-1.497122335288894</v>
       </c>
       <c r="I59">
-        <v>-1.247934316712403</v>
+        <v>-0.6696448191525307</v>
       </c>
       <c r="J59">
-        <v>0.07547096404369455</v>
+        <v>-0.1480490170726664</v>
       </c>
       <c r="K59">
-        <v>-0.5153544800082024</v>
+        <v>0.1990885080772148</v>
       </c>
       <c r="L59">
-        <v>1.367237367222597</v>
+        <v>0.9854276151528297</v>
       </c>
       <c r="M59">
-        <v>0.951065137155752</v>
+        <v>1.130300048284046</v>
       </c>
     </row>
     <row r="60">
@@ -2961,44 +2961,44 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>KAMMINGA_SENESCENCE</t>
+          <t>GOBP_POSITIVE_REGULATION_OF_CELLULAR_SENESCENCE</t>
         </is>
       </c>
       <c r="B61">
-        <v>1.111027647118721</v>
+        <v>-1.364787107537137</v>
       </c>
       <c r="C61">
-        <v>-0.2975745441466948</v>
+        <v>-0.8708796600129045</v>
       </c>
       <c r="D61">
-        <v>1.361458043616241</v>
+        <v>0.1049892474647002</v>
       </c>
       <c r="E61">
-        <v>-0.7280439805049908</v>
+        <v>1.364819788231777</v>
       </c>
       <c r="F61">
-        <v>-0.3721939086084353</v>
+        <v>0.708428435607024</v>
       </c>
       <c r="G61">
-        <v>-1.074673257474841</v>
+        <v>0.05742929624654035</v>
       </c>
       <c r="H61">
-        <v>1.471225630556525</v>
+        <v>-0.6304846717014383</v>
       </c>
       <c r="I61">
-        <v>-0.405441963113315</v>
+        <v>-1.247934316712403</v>
       </c>
       <c r="J61">
-        <v>0.7292611432843187</v>
+        <v>0.07547096404369455</v>
       </c>
       <c r="K61">
-        <v>-0.7714059982495033</v>
+        <v>-0.5153544800082024</v>
       </c>
       <c r="L61">
-        <v>0.202430102019481</v>
+        <v>1.367237367222597</v>
       </c>
       <c r="M61">
-        <v>-1.226068914497507</v>
+        <v>0.951065137155752</v>
       </c>
     </row>
   </sheetData>

</xml_diff>